<commit_message>
feat: implement RSVP management system with detailed dialogs and hooks
- Add RsvpDetailDialog for viewing RSVP request details.
- Implement RsvpRejectDialog for rejecting RSVP requests with optional reason.
- Create RsvpRequestsPage to manage and display RSVP requests with filtering and statistics.
- Introduce RsvpStatsCards to show counts of RSVP statuses.
- Develop RsvpTable for displaying RSVP requests in a tabular format with actions.
- Add hooks for fetching and managing RSVP requests and pending counts.
- Create data structures for RSVP requests and validation schemas.
- Implement server-side session management and authentication checks.
- Update guest management to include source tracking for guests.
- Add sample data and JSON files for testing RSVP functionality.
</commit_message>
<xml_diff>
--- a/src/data/guest-list.xlsx
+++ b/src/data/guest-list.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:J11"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -407,6 +407,8 @@
     <col min="6" max="6" width="12.83203125" customWidth="1"/>
     <col min="7" max="7" width="8.83203125" customWidth="1"/>
     <col min="8" max="8" width="40.83203125" customWidth="1"/>
+    <col min="9" max="9" width="14.83203125" customWidth="1"/>
+    <col min="10" max="10" width="24.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -434,10 +436,336 @@
       <c r="H1" t="str">
         <v>Ghi chú</v>
       </c>
+      <c r="I1" t="str">
+        <v>Nguồn</v>
+      </c>
+      <c r="J1" t="str">
+        <v>ID</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Nguyễn Văn Hùng</v>
+      </c>
+      <c r="B2" t="str">
+        <v>0901234567</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Nhà trai</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Họ hàng</v>
+      </c>
+      <c r="E2">
+        <v>4</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Sẽ đến</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Bác ruột chú rể</v>
+      </c>
+      <c r="I2" t="str">
+        <v>MANUAL</v>
+      </c>
+      <c r="J2" t="str">
+        <v>guest-1787084996213-kr0m44nl</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Trần Thị Lan</v>
+      </c>
+      <c r="B3" t="str">
+        <v>0912345678</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Nhà gái</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Họ hàng</v>
+      </c>
+      <c r="E3">
+        <v>3</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Sẽ đến</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
+      <c r="I3" t="str">
+        <v>MANUAL</v>
+      </c>
+      <c r="J3" t="str">
+        <v>guest-1787084996213-3oweqlcl</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Lê Minh Tuấn</v>
+      </c>
+      <c r="B4" t="str">
+        <v>0923456789</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Nhà trai</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Bạn bè</v>
+      </c>
+      <c r="E4">
+        <v>3</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Sẽ đến</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Bạn đại học</v>
+      </c>
+      <c r="I4" t="str">
+        <v>MANUAL</v>
+      </c>
+      <c r="J4" t="str">
+        <v>guest-1787084996213-xn6j3jvq</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Phạm Thu Hà</v>
+      </c>
+      <c r="B5" t="str">
+        <v>0934567890</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Nhà gái</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Đồng nghiệp</v>
+      </c>
+      <c r="E5">
+        <v>5</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Sẽ đến</v>
+      </c>
+      <c r="G5">
+        <v>2</v>
+      </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
+      <c r="I5" t="str">
+        <v>MANUAL</v>
+      </c>
+      <c r="J5" t="str">
+        <v>guest-1787084996213-hdsqgidf</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Hoàng Đức Anh</v>
+      </c>
+      <c r="B6" t="str">
+        <v>0945678901</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Nhà trai</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Đối tác</v>
+      </c>
+      <c r="E6">
+        <v>4</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Sẽ đến</v>
+      </c>
+      <c r="G6">
+        <v>2</v>
+      </c>
+      <c r="H6" t="str">
+        <v/>
+      </c>
+      <c r="I6" t="str">
+        <v>MANUAL</v>
+      </c>
+      <c r="J6" t="str">
+        <v>guest-1787084996213-7bqn8pow</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Vũ Thị Mai</v>
+      </c>
+      <c r="B7" t="str">
+        <v>0956789012</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Nhà gái</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Bạn bè</v>
+      </c>
+      <c r="E7">
+        <v>3</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Sẽ đến</v>
+      </c>
+      <c r="G7">
+        <v>2</v>
+      </c>
+      <c r="H7" t="str">
+        <v>Nhóm bạn thân — bàn 2 đang quá tải, cần chuyển bớt</v>
+      </c>
+      <c r="I7" t="str">
+        <v>MANUAL</v>
+      </c>
+      <c r="J7" t="str">
+        <v>guest-1787084996213-w2l00rmj</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Đặng Quốc Bảo</v>
+      </c>
+      <c r="B8" t="str">
+        <v>0967890123</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Nhà trai</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Hàng xóm</v>
+      </c>
+      <c r="E8">
+        <v>2</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Sẽ đến</v>
+      </c>
+      <c r="G8">
+        <v>3</v>
+      </c>
+      <c r="H8" t="str">
+        <v/>
+      </c>
+      <c r="I8" t="str">
+        <v>MANUAL</v>
+      </c>
+      <c r="J8" t="str">
+        <v>guest-1787084996213-2gj85wff</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Ngô Thị Thu</v>
+      </c>
+      <c r="B9" t="str">
+        <v>0978901234</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Nhà gái</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Khác</v>
+      </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Đã mời</v>
+      </c>
+      <c r="G9" t="str">
+        <v/>
+      </c>
+      <c r="H9" t="str">
+        <v/>
+      </c>
+      <c r="I9" t="str">
+        <v>MANUAL</v>
+      </c>
+      <c r="J9" t="str">
+        <v>guest-1787084996213-8r92yznb</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Bùi Văn Long</v>
+      </c>
+      <c r="B10" t="str">
+        <v>0989012345</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Nhà trai</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Bạn bè</v>
+      </c>
+      <c r="E10">
+        <v>2</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Chưa mời</v>
+      </c>
+      <c r="G10" t="str">
+        <v/>
+      </c>
+      <c r="H10" t="str">
+        <v/>
+      </c>
+      <c r="I10" t="str">
+        <v>MANUAL</v>
+      </c>
+      <c r="J10" t="str">
+        <v>guest-1787084996213-enw3w1zk</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Đỗ Thị Hoa</v>
+      </c>
+      <c r="B11" t="str">
+        <v>0990123456</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Nhà gái</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Họ hàng</v>
+      </c>
+      <c r="E11">
+        <v>1</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Không đến</v>
+      </c>
+      <c r="G11" t="str">
+        <v/>
+      </c>
+      <c r="H11" t="str">
+        <v>Bận việc gia đình</v>
+      </c>
+      <c r="I11" t="str">
+        <v>MANUAL</v>
+      </c>
+      <c r="J11" t="str">
+        <v>guest-1787084996213-ey0u39t4</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: update RSVP status and approval details for guest Nguyễn Văn A
</commit_message>
<xml_diff>
--- a/src/data/guest-list.xlsx
+++ b/src/data/guest-list.xlsx
@@ -713,10 +713,10 @@
         <v>Bạn bè</v>
       </c>
       <c r="E10">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F10" t="str">
-        <v>Chưa mời</v>
+        <v>Sẽ đến</v>
       </c>
       <c r="G10" t="str">
         <v/>

</xml_diff>

<commit_message>
fix: update RSVP details for guests and adjust statuses
</commit_message>
<xml_diff>
--- a/src/data/guest-list.xlsx
+++ b/src/data/guest-list.xlsx
@@ -472,7 +472,7 @@
         <v>MANUAL</v>
       </c>
       <c r="J2" t="str">
-        <v>guest-1787084996213-kr0m44nl</v>
+        <v>guest-1787085195433-8kjdhzrx</v>
       </c>
     </row>
     <row r="3">
@@ -504,7 +504,7 @@
         <v>MANUAL</v>
       </c>
       <c r="J3" t="str">
-        <v>guest-1787084996213-3oweqlcl</v>
+        <v>guest-1787085195433-cdkuc1ex</v>
       </c>
     </row>
     <row r="4">
@@ -536,7 +536,7 @@
         <v>MANUAL</v>
       </c>
       <c r="J4" t="str">
-        <v>guest-1787084996213-xn6j3jvq</v>
+        <v>guest-1787085195433-1ej4cizd</v>
       </c>
     </row>
     <row r="5">
@@ -568,7 +568,7 @@
         <v>MANUAL</v>
       </c>
       <c r="J5" t="str">
-        <v>guest-1787084996213-hdsqgidf</v>
+        <v>guest-1787085195433-howitbdk</v>
       </c>
     </row>
     <row r="6">
@@ -600,7 +600,7 @@
         <v>MANUAL</v>
       </c>
       <c r="J6" t="str">
-        <v>guest-1787084996213-7bqn8pow</v>
+        <v>guest-1787085195433-sp0f4ju1</v>
       </c>
     </row>
     <row r="7">
@@ -632,7 +632,7 @@
         <v>MANUAL</v>
       </c>
       <c r="J7" t="str">
-        <v>guest-1787084996213-w2l00rmj</v>
+        <v>guest-1787085195433-hq0g5vle</v>
       </c>
     </row>
     <row r="8">
@@ -664,7 +664,7 @@
         <v>MANUAL</v>
       </c>
       <c r="J8" t="str">
-        <v>guest-1787084996213-2gj85wff</v>
+        <v>guest-1787085195433-1z0kybfe</v>
       </c>
     </row>
     <row r="9">
@@ -696,7 +696,7 @@
         <v>MANUAL</v>
       </c>
       <c r="J9" t="str">
-        <v>guest-1787084996213-8r92yznb</v>
+        <v>guest-1787085195433-v4b0x2ue</v>
       </c>
     </row>
     <row r="10">
@@ -713,10 +713,10 @@
         <v>Bạn bè</v>
       </c>
       <c r="E10">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F10" t="str">
-        <v>Sẽ đến</v>
+        <v>Chưa mời</v>
       </c>
       <c r="G10" t="str">
         <v/>
@@ -728,7 +728,7 @@
         <v>MANUAL</v>
       </c>
       <c r="J10" t="str">
-        <v>guest-1787084996213-enw3w1zk</v>
+        <v>guest-1787085195433-fw6dp02c</v>
       </c>
     </row>
     <row r="11">
@@ -760,7 +760,7 @@
         <v>MANUAL</v>
       </c>
       <c r="J11" t="str">
-        <v>guest-1787084996213-ey0u39t4</v>
+        <v>guest-1787085195433-elpx0ocp</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: enhance RSVP management with creation mode and update sidebar navigation
</commit_message>
<xml_diff>
--- a/src/data/guest-list.xlsx
+++ b/src/data/guest-list.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J12"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -763,9 +763,41 @@
         <v>guest-1787085195433-elpx0ocp</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Trần Thị B</v>
+      </c>
+      <c r="B12" t="str">
+        <v>0922333444</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Nhà trai</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Họ hàng</v>
+      </c>
+      <c r="E12">
+        <v>1</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Sẽ đến</v>
+      </c>
+      <c r="G12" t="str">
+        <v/>
+      </c>
+      <c r="H12" t="str">
+        <v/>
+      </c>
+      <c r="I12" t="str">
+        <v>RSVP</v>
+      </c>
+      <c r="J12" t="str">
+        <v>guest-1787085912197-uydcmkst</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J12"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: enhance RSVP functionality and admin UI
- Updated RSVPSection to pre-select guest side based on invitation side.
- Improved SmoothScroll to disable smooth scrolling on admin routes.
- Enhanced AdminSidebar with mobile drawer and bottom tab navigation.
- Added InviteLinkGenerator component for creating invitation links.
- Refactored GuestTable to display guests as cards on mobile.
- Improved RsvpTable with mobile-friendly layout and request actions.
- Updated Dialog component for better mobile experience.
- Cleaned up weddingData by removing unused lunar date label.
- Added empty state components for better user feedback in tables.
- Updated global styles to include tailwindcss-animate plugin.
- Modified guest list and RSVP requests data for testing.
</commit_message>
<xml_diff>
--- a/src/data/guest-list.xlsx
+++ b/src/data/guest-list.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:J2"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -445,10 +445,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Nguyễn Văn Hùng</v>
+        <v/>
       </c>
       <c r="B2" t="str">
-        <v>0901234567</v>
+        <v/>
       </c>
       <c r="C2" t="str">
         <v>Nhà trai</v>
@@ -457,347 +457,27 @@
         <v>Họ hàng</v>
       </c>
       <c r="E2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F2" t="str">
-        <v>Sẽ đến</v>
-      </c>
-      <c r="G2">
-        <v>1</v>
+        <v>Chưa mời</v>
+      </c>
+      <c r="G2" t="str">
+        <v/>
       </c>
       <c r="H2" t="str">
-        <v>Bác ruột chú rể</v>
+        <v/>
       </c>
       <c r="I2" t="str">
         <v>MANUAL</v>
       </c>
       <c r="J2" t="str">
-        <v>guest-1787085195433-8kjdhzrx</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Trần Thị Lan</v>
-      </c>
-      <c r="B3" t="str">
-        <v>0912345678</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Nhà gái</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Họ hàng</v>
-      </c>
-      <c r="E3">
-        <v>3</v>
-      </c>
-      <c r="F3" t="str">
-        <v>Sẽ đến</v>
-      </c>
-      <c r="G3">
-        <v>1</v>
-      </c>
-      <c r="H3" t="str">
-        <v/>
-      </c>
-      <c r="I3" t="str">
-        <v>MANUAL</v>
-      </c>
-      <c r="J3" t="str">
-        <v>guest-1787085195433-cdkuc1ex</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Lê Minh Tuấn</v>
-      </c>
-      <c r="B4" t="str">
-        <v>0923456789</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Nhà trai</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Bạn bè</v>
-      </c>
-      <c r="E4">
-        <v>3</v>
-      </c>
-      <c r="F4" t="str">
-        <v>Sẽ đến</v>
-      </c>
-      <c r="G4">
-        <v>1</v>
-      </c>
-      <c r="H4" t="str">
-        <v>Bạn đại học</v>
-      </c>
-      <c r="I4" t="str">
-        <v>MANUAL</v>
-      </c>
-      <c r="J4" t="str">
-        <v>guest-1787085195433-1ej4cizd</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Phạm Thu Hà</v>
-      </c>
-      <c r="B5" t="str">
-        <v>0934567890</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Nhà gái</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Đồng nghiệp</v>
-      </c>
-      <c r="E5">
-        <v>5</v>
-      </c>
-      <c r="F5" t="str">
-        <v>Sẽ đến</v>
-      </c>
-      <c r="G5">
-        <v>2</v>
-      </c>
-      <c r="H5" t="str">
-        <v/>
-      </c>
-      <c r="I5" t="str">
-        <v>MANUAL</v>
-      </c>
-      <c r="J5" t="str">
-        <v>guest-1787085195433-howitbdk</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Hoàng Đức Anh</v>
-      </c>
-      <c r="B6" t="str">
-        <v>0945678901</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Nhà trai</v>
-      </c>
-      <c r="D6" t="str">
-        <v>Đối tác</v>
-      </c>
-      <c r="E6">
-        <v>4</v>
-      </c>
-      <c r="F6" t="str">
-        <v>Sẽ đến</v>
-      </c>
-      <c r="G6">
-        <v>2</v>
-      </c>
-      <c r="H6" t="str">
-        <v/>
-      </c>
-      <c r="I6" t="str">
-        <v>MANUAL</v>
-      </c>
-      <c r="J6" t="str">
-        <v>guest-1787085195433-sp0f4ju1</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>Vũ Thị Mai</v>
-      </c>
-      <c r="B7" t="str">
-        <v>0956789012</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Nhà gái</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Bạn bè</v>
-      </c>
-      <c r="E7">
-        <v>3</v>
-      </c>
-      <c r="F7" t="str">
-        <v>Sẽ đến</v>
-      </c>
-      <c r="G7">
-        <v>2</v>
-      </c>
-      <c r="H7" t="str">
-        <v>Nhóm bạn thân — bàn 2 đang quá tải, cần chuyển bớt</v>
-      </c>
-      <c r="I7" t="str">
-        <v>MANUAL</v>
-      </c>
-      <c r="J7" t="str">
-        <v>guest-1787085195433-hq0g5vle</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Đặng Quốc Bảo</v>
-      </c>
-      <c r="B8" t="str">
-        <v>0967890123</v>
-      </c>
-      <c r="C8" t="str">
-        <v>Nhà trai</v>
-      </c>
-      <c r="D8" t="str">
-        <v>Hàng xóm</v>
-      </c>
-      <c r="E8">
-        <v>2</v>
-      </c>
-      <c r="F8" t="str">
-        <v>Sẽ đến</v>
-      </c>
-      <c r="G8">
-        <v>3</v>
-      </c>
-      <c r="H8" t="str">
-        <v/>
-      </c>
-      <c r="I8" t="str">
-        <v>MANUAL</v>
-      </c>
-      <c r="J8" t="str">
-        <v>guest-1787085195433-1z0kybfe</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>Ngô Thị Thu</v>
-      </c>
-      <c r="B9" t="str">
-        <v>0978901234</v>
-      </c>
-      <c r="C9" t="str">
-        <v>Nhà gái</v>
-      </c>
-      <c r="D9" t="str">
-        <v>Khác</v>
-      </c>
-      <c r="E9">
-        <v>1</v>
-      </c>
-      <c r="F9" t="str">
-        <v>Đã mời</v>
-      </c>
-      <c r="G9" t="str">
-        <v/>
-      </c>
-      <c r="H9" t="str">
-        <v/>
-      </c>
-      <c r="I9" t="str">
-        <v>MANUAL</v>
-      </c>
-      <c r="J9" t="str">
-        <v>guest-1787085195433-v4b0x2ue</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>Bùi Văn Long</v>
-      </c>
-      <c r="B10" t="str">
-        <v>0989012345</v>
-      </c>
-      <c r="C10" t="str">
-        <v>Nhà trai</v>
-      </c>
-      <c r="D10" t="str">
-        <v>Bạn bè</v>
-      </c>
-      <c r="E10">
-        <v>2</v>
-      </c>
-      <c r="F10" t="str">
-        <v>Chưa mời</v>
-      </c>
-      <c r="G10" t="str">
-        <v/>
-      </c>
-      <c r="H10" t="str">
-        <v/>
-      </c>
-      <c r="I10" t="str">
-        <v>MANUAL</v>
-      </c>
-      <c r="J10" t="str">
-        <v>guest-1787085195433-fw6dp02c</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>Đỗ Thị Hoa</v>
-      </c>
-      <c r="B11" t="str">
-        <v>0990123456</v>
-      </c>
-      <c r="C11" t="str">
-        <v>Nhà gái</v>
-      </c>
-      <c r="D11" t="str">
-        <v>Họ hàng</v>
-      </c>
-      <c r="E11">
-        <v>1</v>
-      </c>
-      <c r="F11" t="str">
-        <v>Không đến</v>
-      </c>
-      <c r="G11" t="str">
-        <v/>
-      </c>
-      <c r="H11" t="str">
-        <v>Bận việc gia đình</v>
-      </c>
-      <c r="I11" t="str">
-        <v>MANUAL</v>
-      </c>
-      <c r="J11" t="str">
-        <v>guest-1787085195433-elpx0ocp</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>Trần Thị B</v>
-      </c>
-      <c r="B12" t="str">
-        <v>0922333444</v>
-      </c>
-      <c r="C12" t="str">
-        <v>Nhà trai</v>
-      </c>
-      <c r="D12" t="str">
-        <v>Họ hàng</v>
-      </c>
-      <c r="E12">
-        <v>1</v>
-      </c>
-      <c r="F12" t="str">
-        <v>Sẽ đến</v>
-      </c>
-      <c r="G12" t="str">
-        <v/>
-      </c>
-      <c r="H12" t="str">
-        <v/>
-      </c>
-      <c r="I12" t="str">
-        <v>RSVP</v>
-      </c>
-      <c r="J12" t="str">
-        <v>guest-1787085912197-uydcmkst</v>
+        <v>ed8c17d6-fa84-40dc-9ba8-02d16153b156</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>